<commit_message>
Add multiple test result CSV files for SAVAGE loss function experiments
- Created new CSV files containing training and testing results for various configurations of the LMC model using the SAVAGE loss function.
- Each file includes parameters such as sample size, beta values, BCE losses, and EMA statistics.
- The experiments cover different selected classes from the CIFAR-100 dataset and various random seeds.
- Summary sections in each file detail the model configuration and performance metrics.
</commit_message>
<xml_diff>
--- a/table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
+++ b/table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,97 @@
       <c r="G1" t="inlineStr">
         <is>
           <t xml:space="preserve">Mean 01 test  loss at infinity </t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[41,42]</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.2505652892850422</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1264586674508169</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.001333775778687512</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1046865051246339</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.001000000047497451</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.135000005364418</v>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Summary:</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meta-learning experiment summary
+  - Table path: table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
+  - Test mode: True
+  - Dataset type: cifar100
+  - Random labels: 0
+  - Number of new pairs requested: 25
+  - Pair sampling seed: 42
+  - Planned pairs: [[41, 42], [9, 91], [50, 65], [1, 70], [15, 78], [10, 73], [55, 56], [45, 72], [48, 92], [37, 76], [21, 30], [32, 96], [49, 80], [26, 83], [33, 87], [8, 47], [59, 63], [44, 74], [52, 98], [12, 85], [23, 36], [39, 40], [18, 66], [60, 61], [7, 34]]
+  - ULA beta values: [128, 1000]
+  - GD beta proxy: [1000000]
+  - Seeds: [42]
+  - Dataset seed: 42
+  - Use same dataset across seeds: True
+  - Loss: SAVAGE
+  - Hidden layers: 1
+  - Width: 500
+  - n_train_per_group: 500
+  - n_test_per_group: 100
+  - batch_size: 1000
+  - a0: {0: 0.01, 128: 0.01, 1000: 0.01, 1000000: 0.01}
+  - sigma_gauss_prior: 5.0
+  - min_steps: 2000
+  - min_steps_first_beta: 4000
+  - alpha_average: 0.01
+  - alpha_stop: 0.00025
+  - eta: 36
+  - eps: -1e-07
+</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new script to recover and append meta-learning table rows from CSV outputs
</commit_message>
<xml_diff>
--- a/table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
+++ b/table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,70 +478,504 @@
         <v>0.135000005364418</v>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Summary:</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Meta-learning experiment summary
-  - Table path: table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
-  - Test mode: True
-  - Dataset type: cifar100
-  - Random labels: 0
-  - Number of new pairs requested: 25
-  - Pair sampling seed: 42
-  - Planned pairs: [[41, 42], [9, 91], [50, 65], [1, 70], [15, 78], [10, 73], [55, 56], [45, 72], [48, 92], [37, 76], [21, 30], [32, 96], [49, 80], [26, 83], [33, 87], [8, 47], [59, 63], [44, 74], [52, 98], [12, 85], [23, 36], [39, 40], [18, 66], [60, 61], [7, 34]]
-  - ULA beta values: [128, 1000]
-  - GD beta proxy: [1000000]
-  - Seeds: [42]
-  - Dataset seed: 42
-  - Use same dataset across seeds: True
-  - Loss: SAVAGE
-  - Hidden layers: 1
-  - Width: 500
-  - n_train_per_group: 500
-  - n_test_per_group: 100
-  - batch_size: 1000
-  - a0: {0: 0.01, 128: 0.01, 1000: 0.01, 1000000: 0.01}
-  - sigma_gauss_prior: 5.0
-  - min_steps: 2000
-  - min_steps_first_beta: 4000
-  - alpha_average: 0.01
-  - alpha_stop: 0.00025
-  - eta: 36
-  - eps: -1e-07
-</t>
-        </is>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>[0,9]</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.2311992686835836</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.07512737888835212</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0002442803093576108</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0677440838576272</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.09000000357627869</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>[1,22]</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.2452578392734399</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1292026808031547</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0003422379562630142</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.09723682222804662</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.1207692284996693</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>[2,92]</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.2445742472936217</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.1355087065004155</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.003256296649152505</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1185720738824122</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.003000000026077032</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.1401733469588517</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>[3,31]</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.4124708696439868</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.2100305560469299</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0006090271105693133</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.2234299902370704</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.2935884706029526</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>[7,50]</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.3443813122784051</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.1773066568166795</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.001600827755614997</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.1730991566090016</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.001000000047497451</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.2404806781247737</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>[10,73]</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.2046919793098944</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.09430422062136473</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.001316792015001469</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.08873965694017551</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.001000000047497451</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.1150000020861626</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>[11,26]</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3801154483884966</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.1848291959238424</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.0004201562931747183</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1475635213742074</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1994061947936644</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>[14,75]</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3723091159126285</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.1485224848845629</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0003320951527719734</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1299004275752026</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.1844140810833367</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>[15,78]</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.3909887821620662</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.1882533437172346</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.00148642952196068</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1845553104130532</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.001000000047497451</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.2452860311585</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[19,59]</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.265013470831169</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.1159702019687404</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.002302729525006638</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.1060768147680982</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.002000000094994903</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.1550000011920929</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>[21,30]</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1530180891594591</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.04931872547800942</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.0002052212977054427</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.02596300146886856</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.02999999932944775</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>[32,96]</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3113539990030819</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.1332556925017166</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.001489818373561487</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.1179592455911405</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.001000000047497451</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.1632842659863747</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>[33,87]</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2649666342711103</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.1256015914671992</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.001392873332953054</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.1208211544772657</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.001000000047497451</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1500000059604645</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>[34,58]</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2867710706185738</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1076944708124315</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.0002423465577903793</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.08921744282080867</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.1099999994039536</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>[37,76]</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.2568527583005218</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.1260425489485442</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.001313697414927604</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.08822127379856798</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.001000000047497451</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.1258871282755467</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>[40,98]</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.3297037731891298</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1716934776238455</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.0004006391519683717</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.1574959574077893</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.2150000035762787</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>[45,72]</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.3121707689714034</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.1558021337502922</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.001461012264580873</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.1687240328287251</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.001000000047497451</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.2249999940395355</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>[49,80]</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.1354204012785246</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.0536077593460269</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.0002312821269669839</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.04419732523645285</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.03999999910593033</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>[55,56]</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.3222211563261425</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.1464295812854618</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.0004434085455111959</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.1155414478853612</v>
+      </c>
+      <c r="F21" t="n">
+        <v>7.879882319315714e-05</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.1519057890260188</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>[57,71]</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.1358822462917492</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.04770399732657415</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.0001982284945809077</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.04620583054217815</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.05499999970197678</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add new CSV files for SAVAGE loss function experiments and update sampling seed
</commit_message>
<xml_diff>
--- a/table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
+++ b/table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -978,6 +978,18 @@
         <v>0.05499999970197678</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>[62,68]</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add CSV files for SAVAGE loss function experiments with varying beta values
- Created multiple CSV files documenting the results of experiments using the SAVAGE loss function on the CIFAR-100 dataset.
- Each file includes metrics such as BCE Train/Test, EMA losses, and gradient norms for different beta values.
- Updated summary sections to reflect the parameters used in each experiment, including device, network architecture, learning rates, and training details.
- Added a new Excel file to track meta-learning results associated with the experiments.
</commit_message>
<xml_diff>
--- a/table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
+++ b/table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -984,9 +984,281 @@
           <t>[62,68]</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" t="n">
+        <v>0.1295012187080731</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.03598911725025162</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.0001377629007389235</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.03183543962533922</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.03614091451719362</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>[8,51]</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.2532637857056322</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.1259978745780068</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.0003035037279541545</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.1036843115291966</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.1400000005960464</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>[60,79]</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.1192555010048483</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.04914622507104684</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.0003054199962956257</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.03663718916079458</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.05350211614270621</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>[16,46]</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.322617482186438</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.192360777675677</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.0004604328659534357</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.167575666482183</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.1996811699690723</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>[27,44]</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.4100246841365187</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.2320266476345171</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.0008804690439529423</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.2795214612835209</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.3677093765189835</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>[6,69]</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.1949760208485167</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.0627587462970056</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.0002478219586233731</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.05867295239316216</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.07500000298023224</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>[39,70]</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.2349414412001112</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.1014982836323501</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.000251880544383431</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.06901741464631546</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.09000000357627869</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>[24,77]</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.2126781450647555</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.1323032025474663</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.004138386995363541</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.09801316777613134</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.003400014221426505</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.127263765547486</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>[35,52]</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.127485979559937</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.03046894737278476</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.0001254026363323162</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.01680271922800508</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.02500000037252903</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>[94,99]</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Summary:</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meta-learning experiment summary
+  - Table path: table_meta_learning_CCL1W500ULA_GD1kLR001SAVAGE.xlsx
+  - Test mode: True
+  - Dataset type: cifar100
+  - Random labels: 0
+  - Number of new pairs requested: 25
+  - Pair sampling seed: 52
+  - Planned pairs: sampled online one-by-one
+  - ULA beta values: [128, 1000]
+  - GD beta proxy: [1000000]
+  - Seeds: [42]
+  - Dataset seed: 42
+  - Use same dataset across seeds: True
+  - Loss: SAVAGE
+  - Hidden layers: 1
+  - Width: 500
+  - n_train_per_group: 500
+  - n_test_per_group: 100
+  - batch_size: 1000
+  - a0: {0: 0.01, 128: 0.01, 1000: 0.01, 1000000: 0.01}
+  - sigma_gauss_prior: 5.0
+  - min_steps: 2000
+  - min_steps_first_beta: 4000
+  - alpha_average: 0.01
+  - alpha_stop: 0.00025
+  - eta: 36
+  - eps: -1e-07
+</t>
         </is>
       </c>
     </row>

</xml_diff>